<commit_message>
Add head/short keyword terms (bare category words) to research list
Adds 67 head terms (single-word like crm/invoicing/scheduling, two-word
category concepts, and short modifiers like best crm/free crm/what is crm)
so the research captures the highest-volume broad terms that set each
category's ceiling. Workbook now totals 418 tagged keywords.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WuJPSeeTeWNKm9gY9rLHNX
</commit_message>
<xml_diff>
--- a/Demand_Keyword_Research_List.xlsx
+++ b/Demand_Keyword_Research_List.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paste list (flat)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keyword Research List'!$A$1:$O$352</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keyword Research List'!$A$1:$O$419</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O352"/>
+  <dimension ref="A1:O419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14393,8 +14393,2621 @@
       <c r="N352" s="7" t="inlineStr"/>
       <c r="O352" s="7" t="inlineStr"/>
     </row>
+    <row r="353">
+      <c r="A353" s="5" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" s="6" t="inlineStr">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="C353" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D353" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E353" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F353" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G353" s="7" t="inlineStr"/>
+      <c r="H353" s="7" t="inlineStr"/>
+      <c r="I353" s="7" t="inlineStr"/>
+      <c r="J353" s="7" t="inlineStr"/>
+      <c r="K353" s="7" t="inlineStr"/>
+      <c r="L353" s="7" t="inlineStr"/>
+      <c r="M353" s="7" t="inlineStr"/>
+      <c r="N353" s="7" t="inlineStr"/>
+      <c r="O353" s="7" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="5" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" s="6" t="inlineStr">
+        <is>
+          <t>invoicing</t>
+        </is>
+      </c>
+      <c r="C354" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D354" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E354" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F354" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G354" s="7" t="inlineStr"/>
+      <c r="H354" s="7" t="inlineStr"/>
+      <c r="I354" s="7" t="inlineStr"/>
+      <c r="J354" s="7" t="inlineStr"/>
+      <c r="K354" s="7" t="inlineStr"/>
+      <c r="L354" s="7" t="inlineStr"/>
+      <c r="M354" s="7" t="inlineStr"/>
+      <c r="N354" s="7" t="inlineStr"/>
+      <c r="O354" s="7" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="5" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" s="6" t="inlineStr">
+        <is>
+          <t>invoice</t>
+        </is>
+      </c>
+      <c r="C355" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D355" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E355" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F355" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G355" s="7" t="inlineStr"/>
+      <c r="H355" s="7" t="inlineStr"/>
+      <c r="I355" s="7" t="inlineStr"/>
+      <c r="J355" s="7" t="inlineStr"/>
+      <c r="K355" s="7" t="inlineStr"/>
+      <c r="L355" s="7" t="inlineStr"/>
+      <c r="M355" s="7" t="inlineStr"/>
+      <c r="N355" s="7" t="inlineStr"/>
+      <c r="O355" s="7" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="5" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" s="6" t="inlineStr">
+        <is>
+          <t>scheduling</t>
+        </is>
+      </c>
+      <c r="C356" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D356" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E356" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F356" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G356" s="7" t="inlineStr"/>
+      <c r="H356" s="7" t="inlineStr"/>
+      <c r="I356" s="7" t="inlineStr"/>
+      <c r="J356" s="7" t="inlineStr"/>
+      <c r="K356" s="7" t="inlineStr"/>
+      <c r="L356" s="7" t="inlineStr"/>
+      <c r="M356" s="7" t="inlineStr"/>
+      <c r="N356" s="7" t="inlineStr"/>
+      <c r="O356" s="7" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="5" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" s="6" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+      <c r="C357" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D357" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E357" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F357" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G357" s="7" t="inlineStr"/>
+      <c r="H357" s="7" t="inlineStr"/>
+      <c r="I357" s="7" t="inlineStr"/>
+      <c r="J357" s="7" t="inlineStr"/>
+      <c r="K357" s="7" t="inlineStr"/>
+      <c r="L357" s="7" t="inlineStr"/>
+      <c r="M357" s="7" t="inlineStr"/>
+      <c r="N357" s="7" t="inlineStr"/>
+      <c r="O357" s="7" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="5" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" s="6" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C358" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D358" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E358" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F358" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G358" s="7" t="inlineStr"/>
+      <c r="H358" s="7" t="inlineStr"/>
+      <c r="I358" s="7" t="inlineStr"/>
+      <c r="J358" s="7" t="inlineStr"/>
+      <c r="K358" s="7" t="inlineStr"/>
+      <c r="L358" s="7" t="inlineStr"/>
+      <c r="M358" s="7" t="inlineStr"/>
+      <c r="N358" s="7" t="inlineStr"/>
+      <c r="O358" s="7" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="5" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" s="6" t="inlineStr">
+        <is>
+          <t>proposal</t>
+        </is>
+      </c>
+      <c r="C359" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D359" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E359" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F359" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G359" s="7" t="inlineStr"/>
+      <c r="H359" s="7" t="inlineStr"/>
+      <c r="I359" s="7" t="inlineStr"/>
+      <c r="J359" s="7" t="inlineStr"/>
+      <c r="K359" s="7" t="inlineStr"/>
+      <c r="L359" s="7" t="inlineStr"/>
+      <c r="M359" s="7" t="inlineStr"/>
+      <c r="N359" s="7" t="inlineStr"/>
+      <c r="O359" s="7" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="5" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="6" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C360" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D360" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E360" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F360" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G360" s="7" t="inlineStr"/>
+      <c r="H360" s="7" t="inlineStr"/>
+      <c r="I360" s="7" t="inlineStr"/>
+      <c r="J360" s="7" t="inlineStr"/>
+      <c r="K360" s="7" t="inlineStr"/>
+      <c r="L360" s="7" t="inlineStr"/>
+      <c r="M360" s="7" t="inlineStr"/>
+      <c r="N360" s="7" t="inlineStr"/>
+      <c r="O360" s="7" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="6" t="inlineStr">
+        <is>
+          <t>leads</t>
+        </is>
+      </c>
+      <c r="C361" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D361" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E361" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F361" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G361" s="7" t="inlineStr"/>
+      <c r="H361" s="7" t="inlineStr"/>
+      <c r="I361" s="7" t="inlineStr"/>
+      <c r="J361" s="7" t="inlineStr"/>
+      <c r="K361" s="7" t="inlineStr"/>
+      <c r="L361" s="7" t="inlineStr"/>
+      <c r="M361" s="7" t="inlineStr"/>
+      <c r="N361" s="7" t="inlineStr"/>
+      <c r="O361" s="7" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="5" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="6" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="C362" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D362" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E362" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F362" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G362" s="7" t="inlineStr"/>
+      <c r="H362" s="7" t="inlineStr"/>
+      <c r="I362" s="7" t="inlineStr"/>
+      <c r="J362" s="7" t="inlineStr"/>
+      <c r="K362" s="7" t="inlineStr"/>
+      <c r="L362" s="7" t="inlineStr"/>
+      <c r="M362" s="7" t="inlineStr"/>
+      <c r="N362" s="7" t="inlineStr"/>
+      <c r="O362" s="7" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="6" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+      <c r="C363" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D363" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E363" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F363" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G363" s="7" t="inlineStr"/>
+      <c r="H363" s="7" t="inlineStr"/>
+      <c r="I363" s="7" t="inlineStr"/>
+      <c r="J363" s="7" t="inlineStr"/>
+      <c r="K363" s="7" t="inlineStr"/>
+      <c r="L363" s="7" t="inlineStr"/>
+      <c r="M363" s="7" t="inlineStr"/>
+      <c r="N363" s="7" t="inlineStr"/>
+      <c r="O363" s="7" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="5" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="6" t="inlineStr">
+        <is>
+          <t>reporting</t>
+        </is>
+      </c>
+      <c r="C364" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D364" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E364" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F364" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G364" s="7" t="inlineStr"/>
+      <c r="H364" s="7" t="inlineStr"/>
+      <c r="I364" s="7" t="inlineStr"/>
+      <c r="J364" s="7" t="inlineStr"/>
+      <c r="K364" s="7" t="inlineStr"/>
+      <c r="L364" s="7" t="inlineStr"/>
+      <c r="M364" s="7" t="inlineStr"/>
+      <c r="N364" s="7" t="inlineStr"/>
+      <c r="O364" s="7" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="6" t="inlineStr">
+        <is>
+          <t>forms</t>
+        </is>
+      </c>
+      <c r="C365" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D365" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E365" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F365" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G365" s="7" t="inlineStr"/>
+      <c r="H365" s="7" t="inlineStr"/>
+      <c r="I365" s="7" t="inlineStr"/>
+      <c r="J365" s="7" t="inlineStr"/>
+      <c r="K365" s="7" t="inlineStr"/>
+      <c r="L365" s="7" t="inlineStr"/>
+      <c r="M365" s="7" t="inlineStr"/>
+      <c r="N365" s="7" t="inlineStr"/>
+      <c r="O365" s="7" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="6" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+      <c r="C366" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D366" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E366" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F366" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G366" s="7" t="inlineStr"/>
+      <c r="H366" s="7" t="inlineStr"/>
+      <c r="I366" s="7" t="inlineStr"/>
+      <c r="J366" s="7" t="inlineStr"/>
+      <c r="K366" s="7" t="inlineStr"/>
+      <c r="L366" s="7" t="inlineStr"/>
+      <c r="M366" s="7" t="inlineStr"/>
+      <c r="N366" s="7" t="inlineStr"/>
+      <c r="O366" s="7" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="6" t="inlineStr">
+        <is>
+          <t>appointments</t>
+        </is>
+      </c>
+      <c r="C367" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D367" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E367" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F367" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G367" s="7" t="inlineStr"/>
+      <c r="H367" s="7" t="inlineStr"/>
+      <c r="I367" s="7" t="inlineStr"/>
+      <c r="J367" s="7" t="inlineStr"/>
+      <c r="K367" s="7" t="inlineStr"/>
+      <c r="L367" s="7" t="inlineStr"/>
+      <c r="M367" s="7" t="inlineStr"/>
+      <c r="N367" s="7" t="inlineStr"/>
+      <c r="O367" s="7" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="5" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="6" t="inlineStr">
+        <is>
+          <t>quotes</t>
+        </is>
+      </c>
+      <c r="C368" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D368" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E368" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F368" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G368" s="7" t="inlineStr"/>
+      <c r="H368" s="7" t="inlineStr"/>
+      <c r="I368" s="7" t="inlineStr"/>
+      <c r="J368" s="7" t="inlineStr"/>
+      <c r="K368" s="7" t="inlineStr"/>
+      <c r="L368" s="7" t="inlineStr"/>
+      <c r="M368" s="7" t="inlineStr"/>
+      <c r="N368" s="7" t="inlineStr"/>
+      <c r="O368" s="7" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="5" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="6" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="C369" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D369" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F369" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G369" s="7" t="inlineStr"/>
+      <c r="H369" s="7" t="inlineStr"/>
+      <c r="I369" s="7" t="inlineStr"/>
+      <c r="J369" s="7" t="inlineStr"/>
+      <c r="K369" s="7" t="inlineStr"/>
+      <c r="L369" s="7" t="inlineStr"/>
+      <c r="M369" s="7" t="inlineStr"/>
+      <c r="N369" s="7" t="inlineStr"/>
+      <c r="O369" s="7" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="5" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="6" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="C370" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D370" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E370" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F370" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G370" s="7" t="inlineStr"/>
+      <c r="H370" s="7" t="inlineStr"/>
+      <c r="I370" s="7" t="inlineStr"/>
+      <c r="J370" s="7" t="inlineStr"/>
+      <c r="K370" s="7" t="inlineStr"/>
+      <c r="L370" s="7" t="inlineStr"/>
+      <c r="M370" s="7" t="inlineStr"/>
+      <c r="N370" s="7" t="inlineStr"/>
+      <c r="O370" s="7" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="6" t="inlineStr">
+        <is>
+          <t>helpdesk</t>
+        </is>
+      </c>
+      <c r="C371" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D371" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E371" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F371" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G371" s="7" t="inlineStr"/>
+      <c r="H371" s="7" t="inlineStr"/>
+      <c r="I371" s="7" t="inlineStr"/>
+      <c r="J371" s="7" t="inlineStr"/>
+      <c r="K371" s="7" t="inlineStr"/>
+      <c r="L371" s="7" t="inlineStr"/>
+      <c r="M371" s="7" t="inlineStr"/>
+      <c r="N371" s="7" t="inlineStr"/>
+      <c r="O371" s="7" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="5" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="6" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="C372" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D372" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E372" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F372" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G372" s="7" t="inlineStr"/>
+      <c r="H372" s="7" t="inlineStr"/>
+      <c r="I372" s="7" t="inlineStr"/>
+      <c r="J372" s="7" t="inlineStr"/>
+      <c r="K372" s="7" t="inlineStr"/>
+      <c r="L372" s="7" t="inlineStr"/>
+      <c r="M372" s="7" t="inlineStr"/>
+      <c r="N372" s="7" t="inlineStr"/>
+      <c r="O372" s="7" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="5" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="6" t="inlineStr">
+        <is>
+          <t>newsletters</t>
+        </is>
+      </c>
+      <c r="C373" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D373" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E373" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F373" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G373" s="7" t="inlineStr"/>
+      <c r="H373" s="7" t="inlineStr"/>
+      <c r="I373" s="7" t="inlineStr"/>
+      <c r="J373" s="7" t="inlineStr"/>
+      <c r="K373" s="7" t="inlineStr"/>
+      <c r="L373" s="7" t="inlineStr"/>
+      <c r="M373" s="7" t="inlineStr"/>
+      <c r="N373" s="7" t="inlineStr"/>
+      <c r="O373" s="7" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="5" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="6" t="inlineStr">
+        <is>
+          <t>contacts</t>
+        </is>
+      </c>
+      <c r="C374" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D374" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E374" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F374" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G374" s="7" t="inlineStr"/>
+      <c r="H374" s="7" t="inlineStr"/>
+      <c r="I374" s="7" t="inlineStr"/>
+      <c r="J374" s="7" t="inlineStr"/>
+      <c r="K374" s="7" t="inlineStr"/>
+      <c r="L374" s="7" t="inlineStr"/>
+      <c r="M374" s="7" t="inlineStr"/>
+      <c r="N374" s="7" t="inlineStr"/>
+      <c r="O374" s="7" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="5" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="6" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C375" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D375" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E375" s="5" t="inlineStr">
+        <is>
+          <t>Head (single)</t>
+        </is>
+      </c>
+      <c r="F375" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G375" s="7" t="inlineStr"/>
+      <c r="H375" s="7" t="inlineStr"/>
+      <c r="I375" s="7" t="inlineStr"/>
+      <c r="J375" s="7" t="inlineStr"/>
+      <c r="K375" s="7" t="inlineStr"/>
+      <c r="L375" s="7" t="inlineStr"/>
+      <c r="M375" s="7" t="inlineStr"/>
+      <c r="N375" s="7" t="inlineStr"/>
+      <c r="O375" s="7" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="5" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="6" t="inlineStr">
+        <is>
+          <t>client management</t>
+        </is>
+      </c>
+      <c r="C376" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D376" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E376" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F376" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G376" s="7" t="inlineStr"/>
+      <c r="H376" s="7" t="inlineStr"/>
+      <c r="I376" s="7" t="inlineStr"/>
+      <c r="J376" s="7" t="inlineStr"/>
+      <c r="K376" s="7" t="inlineStr"/>
+      <c r="L376" s="7" t="inlineStr"/>
+      <c r="M376" s="7" t="inlineStr"/>
+      <c r="N376" s="7" t="inlineStr"/>
+      <c r="O376" s="7" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="5" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="6" t="inlineStr">
+        <is>
+          <t>project management</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D377" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E377" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F377" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G377" s="7" t="inlineStr"/>
+      <c r="H377" s="7" t="inlineStr"/>
+      <c r="I377" s="7" t="inlineStr"/>
+      <c r="J377" s="7" t="inlineStr"/>
+      <c r="K377" s="7" t="inlineStr"/>
+      <c r="L377" s="7" t="inlineStr"/>
+      <c r="M377" s="7" t="inlineStr"/>
+      <c r="N377" s="7" t="inlineStr"/>
+      <c r="O377" s="7" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="5" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="6" t="inlineStr">
+        <is>
+          <t>lead management</t>
+        </is>
+      </c>
+      <c r="C378" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D378" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E378" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F378" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G378" s="7" t="inlineStr"/>
+      <c r="H378" s="7" t="inlineStr"/>
+      <c r="I378" s="7" t="inlineStr"/>
+      <c r="J378" s="7" t="inlineStr"/>
+      <c r="K378" s="7" t="inlineStr"/>
+      <c r="L378" s="7" t="inlineStr"/>
+      <c r="M378" s="7" t="inlineStr"/>
+      <c r="N378" s="7" t="inlineStr"/>
+      <c r="O378" s="7" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="5" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="6" t="inlineStr">
+        <is>
+          <t>contact management</t>
+        </is>
+      </c>
+      <c r="C379" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D379" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E379" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F379" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G379" s="7" t="inlineStr"/>
+      <c r="H379" s="7" t="inlineStr"/>
+      <c r="I379" s="7" t="inlineStr"/>
+      <c r="J379" s="7" t="inlineStr"/>
+      <c r="K379" s="7" t="inlineStr"/>
+      <c r="L379" s="7" t="inlineStr"/>
+      <c r="M379" s="7" t="inlineStr"/>
+      <c r="N379" s="7" t="inlineStr"/>
+      <c r="O379" s="7" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="6" t="inlineStr">
+        <is>
+          <t>marketing automation</t>
+        </is>
+      </c>
+      <c r="C380" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D380" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E380" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F380" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G380" s="7" t="inlineStr"/>
+      <c r="H380" s="7" t="inlineStr"/>
+      <c r="I380" s="7" t="inlineStr"/>
+      <c r="J380" s="7" t="inlineStr"/>
+      <c r="K380" s="7" t="inlineStr"/>
+      <c r="L380" s="7" t="inlineStr"/>
+      <c r="M380" s="7" t="inlineStr"/>
+      <c r="N380" s="7" t="inlineStr"/>
+      <c r="O380" s="7" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="5" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="6" t="inlineStr">
+        <is>
+          <t>email marketing</t>
+        </is>
+      </c>
+      <c r="C381" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D381" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E381" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F381" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G381" s="7" t="inlineStr"/>
+      <c r="H381" s="7" t="inlineStr"/>
+      <c r="I381" s="7" t="inlineStr"/>
+      <c r="J381" s="7" t="inlineStr"/>
+      <c r="K381" s="7" t="inlineStr"/>
+      <c r="L381" s="7" t="inlineStr"/>
+      <c r="M381" s="7" t="inlineStr"/>
+      <c r="N381" s="7" t="inlineStr"/>
+      <c r="O381" s="7" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="5" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="6" t="inlineStr">
+        <is>
+          <t>appointment scheduling</t>
+        </is>
+      </c>
+      <c r="C382" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D382" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E382" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F382" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G382" s="7" t="inlineStr"/>
+      <c r="H382" s="7" t="inlineStr"/>
+      <c r="I382" s="7" t="inlineStr"/>
+      <c r="J382" s="7" t="inlineStr"/>
+      <c r="K382" s="7" t="inlineStr"/>
+      <c r="L382" s="7" t="inlineStr"/>
+      <c r="M382" s="7" t="inlineStr"/>
+      <c r="N382" s="7" t="inlineStr"/>
+      <c r="O382" s="7" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="5" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="6" t="inlineStr">
+        <is>
+          <t>online scheduling</t>
+        </is>
+      </c>
+      <c r="C383" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D383" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E383" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F383" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G383" s="7" t="inlineStr"/>
+      <c r="H383" s="7" t="inlineStr"/>
+      <c r="I383" s="7" t="inlineStr"/>
+      <c r="J383" s="7" t="inlineStr"/>
+      <c r="K383" s="7" t="inlineStr"/>
+      <c r="L383" s="7" t="inlineStr"/>
+      <c r="M383" s="7" t="inlineStr"/>
+      <c r="N383" s="7" t="inlineStr"/>
+      <c r="O383" s="7" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="5" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" s="6" t="inlineStr">
+        <is>
+          <t>time tracking</t>
+        </is>
+      </c>
+      <c r="C384" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D384" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E384" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F384" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G384" s="7" t="inlineStr"/>
+      <c r="H384" s="7" t="inlineStr"/>
+      <c r="I384" s="7" t="inlineStr"/>
+      <c r="J384" s="7" t="inlineStr"/>
+      <c r="K384" s="7" t="inlineStr"/>
+      <c r="L384" s="7" t="inlineStr"/>
+      <c r="M384" s="7" t="inlineStr"/>
+      <c r="N384" s="7" t="inlineStr"/>
+      <c r="O384" s="7" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="5" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" s="6" t="inlineStr">
+        <is>
+          <t>customer support</t>
+        </is>
+      </c>
+      <c r="C385" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D385" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E385" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F385" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G385" s="7" t="inlineStr"/>
+      <c r="H385" s="7" t="inlineStr"/>
+      <c r="I385" s="7" t="inlineStr"/>
+      <c r="J385" s="7" t="inlineStr"/>
+      <c r="K385" s="7" t="inlineStr"/>
+      <c r="L385" s="7" t="inlineStr"/>
+      <c r="M385" s="7" t="inlineStr"/>
+      <c r="N385" s="7" t="inlineStr"/>
+      <c r="O385" s="7" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" s="6" t="inlineStr">
+        <is>
+          <t>live chat</t>
+        </is>
+      </c>
+      <c r="C386" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D386" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E386" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F386" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G386" s="7" t="inlineStr"/>
+      <c r="H386" s="7" t="inlineStr"/>
+      <c r="I386" s="7" t="inlineStr"/>
+      <c r="J386" s="7" t="inlineStr"/>
+      <c r="K386" s="7" t="inlineStr"/>
+      <c r="L386" s="7" t="inlineStr"/>
+      <c r="M386" s="7" t="inlineStr"/>
+      <c r="N386" s="7" t="inlineStr"/>
+      <c r="O386" s="7" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="5" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" s="6" t="inlineStr">
+        <is>
+          <t>client portal</t>
+        </is>
+      </c>
+      <c r="C387" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D387" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E387" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F387" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G387" s="7" t="inlineStr"/>
+      <c r="H387" s="7" t="inlineStr"/>
+      <c r="I387" s="7" t="inlineStr"/>
+      <c r="J387" s="7" t="inlineStr"/>
+      <c r="K387" s="7" t="inlineStr"/>
+      <c r="L387" s="7" t="inlineStr"/>
+      <c r="M387" s="7" t="inlineStr"/>
+      <c r="N387" s="7" t="inlineStr"/>
+      <c r="O387" s="7" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="5" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" s="6" t="inlineStr">
+        <is>
+          <t>sales pipeline</t>
+        </is>
+      </c>
+      <c r="C388" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D388" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E388" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F388" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G388" s="7" t="inlineStr"/>
+      <c r="H388" s="7" t="inlineStr"/>
+      <c r="I388" s="7" t="inlineStr"/>
+      <c r="J388" s="7" t="inlineStr"/>
+      <c r="K388" s="7" t="inlineStr"/>
+      <c r="L388" s="7" t="inlineStr"/>
+      <c r="M388" s="7" t="inlineStr"/>
+      <c r="N388" s="7" t="inlineStr"/>
+      <c r="O388" s="7" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="5" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" s="6" t="inlineStr">
+        <is>
+          <t>task management</t>
+        </is>
+      </c>
+      <c r="C389" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D389" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E389" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F389" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G389" s="7" t="inlineStr"/>
+      <c r="H389" s="7" t="inlineStr"/>
+      <c r="I389" s="7" t="inlineStr"/>
+      <c r="J389" s="7" t="inlineStr"/>
+      <c r="K389" s="7" t="inlineStr"/>
+      <c r="L389" s="7" t="inlineStr"/>
+      <c r="M389" s="7" t="inlineStr"/>
+      <c r="N389" s="7" t="inlineStr"/>
+      <c r="O389" s="7" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="5" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" s="6" t="inlineStr">
+        <is>
+          <t>work management</t>
+        </is>
+      </c>
+      <c r="C390" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D390" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E390" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F390" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G390" s="7" t="inlineStr"/>
+      <c r="H390" s="7" t="inlineStr"/>
+      <c r="I390" s="7" t="inlineStr"/>
+      <c r="J390" s="7" t="inlineStr"/>
+      <c r="K390" s="7" t="inlineStr"/>
+      <c r="L390" s="7" t="inlineStr"/>
+      <c r="M390" s="7" t="inlineStr"/>
+      <c r="N390" s="7" t="inlineStr"/>
+      <c r="O390" s="7" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="5" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" s="6" t="inlineStr">
+        <is>
+          <t>customer onboarding</t>
+        </is>
+      </c>
+      <c r="C391" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D391" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E391" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F391" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G391" s="7" t="inlineStr"/>
+      <c r="H391" s="7" t="inlineStr"/>
+      <c r="I391" s="7" t="inlineStr"/>
+      <c r="J391" s="7" t="inlineStr"/>
+      <c r="K391" s="7" t="inlineStr"/>
+      <c r="L391" s="7" t="inlineStr"/>
+      <c r="M391" s="7" t="inlineStr"/>
+      <c r="N391" s="7" t="inlineStr"/>
+      <c r="O391" s="7" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="5" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" s="6" t="inlineStr">
+        <is>
+          <t>sales tracking</t>
+        </is>
+      </c>
+      <c r="C392" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D392" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E392" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F392" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G392" s="7" t="inlineStr"/>
+      <c r="H392" s="7" t="inlineStr"/>
+      <c r="I392" s="7" t="inlineStr"/>
+      <c r="J392" s="7" t="inlineStr"/>
+      <c r="K392" s="7" t="inlineStr"/>
+      <c r="L392" s="7" t="inlineStr"/>
+      <c r="M392" s="7" t="inlineStr"/>
+      <c r="N392" s="7" t="inlineStr"/>
+      <c r="O392" s="7" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="5" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" s="6" t="inlineStr">
+        <is>
+          <t>deal pipeline</t>
+        </is>
+      </c>
+      <c r="C393" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D393" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E393" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F393" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G393" s="7" t="inlineStr"/>
+      <c r="H393" s="7" t="inlineStr"/>
+      <c r="I393" s="7" t="inlineStr"/>
+      <c r="J393" s="7" t="inlineStr"/>
+      <c r="K393" s="7" t="inlineStr"/>
+      <c r="L393" s="7" t="inlineStr"/>
+      <c r="M393" s="7" t="inlineStr"/>
+      <c r="N393" s="7" t="inlineStr"/>
+      <c r="O393" s="7" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="5" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" s="6" t="inlineStr">
+        <is>
+          <t>business management</t>
+        </is>
+      </c>
+      <c r="C394" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D394" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E394" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F394" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G394" s="7" t="inlineStr"/>
+      <c r="H394" s="7" t="inlineStr"/>
+      <c r="I394" s="7" t="inlineStr"/>
+      <c r="J394" s="7" t="inlineStr"/>
+      <c r="K394" s="7" t="inlineStr"/>
+      <c r="L394" s="7" t="inlineStr"/>
+      <c r="M394" s="7" t="inlineStr"/>
+      <c r="N394" s="7" t="inlineStr"/>
+      <c r="O394" s="7" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="5" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" s="6" t="inlineStr">
+        <is>
+          <t>client tracking</t>
+        </is>
+      </c>
+      <c r="C395" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D395" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E395" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F395" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G395" s="7" t="inlineStr"/>
+      <c r="H395" s="7" t="inlineStr"/>
+      <c r="I395" s="7" t="inlineStr"/>
+      <c r="J395" s="7" t="inlineStr"/>
+      <c r="K395" s="7" t="inlineStr"/>
+      <c r="L395" s="7" t="inlineStr"/>
+      <c r="M395" s="7" t="inlineStr"/>
+      <c r="N395" s="7" t="inlineStr"/>
+      <c r="O395" s="7" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="5" t="n">
+        <v>395</v>
+      </c>
+      <c r="B396" s="6" t="inlineStr">
+        <is>
+          <t>lead tracking</t>
+        </is>
+      </c>
+      <c r="C396" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D396" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E396" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F396" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G396" s="7" t="inlineStr"/>
+      <c r="H396" s="7" t="inlineStr"/>
+      <c r="I396" s="7" t="inlineStr"/>
+      <c r="J396" s="7" t="inlineStr"/>
+      <c r="K396" s="7" t="inlineStr"/>
+      <c r="L396" s="7" t="inlineStr"/>
+      <c r="M396" s="7" t="inlineStr"/>
+      <c r="N396" s="7" t="inlineStr"/>
+      <c r="O396" s="7" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="5" t="n">
+        <v>396</v>
+      </c>
+      <c r="B397" s="6" t="inlineStr">
+        <is>
+          <t>sales automation</t>
+        </is>
+      </c>
+      <c r="C397" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D397" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E397" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F397" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G397" s="7" t="inlineStr"/>
+      <c r="H397" s="7" t="inlineStr"/>
+      <c r="I397" s="7" t="inlineStr"/>
+      <c r="J397" s="7" t="inlineStr"/>
+      <c r="K397" s="7" t="inlineStr"/>
+      <c r="L397" s="7" t="inlineStr"/>
+      <c r="M397" s="7" t="inlineStr"/>
+      <c r="N397" s="7" t="inlineStr"/>
+      <c r="O397" s="7" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="5" t="n">
+        <v>397</v>
+      </c>
+      <c r="B398" s="6" t="inlineStr">
+        <is>
+          <t>email automation</t>
+        </is>
+      </c>
+      <c r="C398" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D398" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E398" s="5" t="inlineStr">
+        <is>
+          <t>Head (two-word)</t>
+        </is>
+      </c>
+      <c r="F398" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G398" s="7" t="inlineStr"/>
+      <c r="H398" s="7" t="inlineStr"/>
+      <c r="I398" s="7" t="inlineStr"/>
+      <c r="J398" s="7" t="inlineStr"/>
+      <c r="K398" s="7" t="inlineStr"/>
+      <c r="L398" s="7" t="inlineStr"/>
+      <c r="M398" s="7" t="inlineStr"/>
+      <c r="N398" s="7" t="inlineStr"/>
+      <c r="O398" s="7" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="5" t="n">
+        <v>398</v>
+      </c>
+      <c r="B399" s="6" t="inlineStr">
+        <is>
+          <t>crm app</t>
+        </is>
+      </c>
+      <c r="C399" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D399" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E399" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F399" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G399" s="7" t="inlineStr"/>
+      <c r="H399" s="7" t="inlineStr"/>
+      <c r="I399" s="7" t="inlineStr"/>
+      <c r="J399" s="7" t="inlineStr"/>
+      <c r="K399" s="7" t="inlineStr"/>
+      <c r="L399" s="7" t="inlineStr"/>
+      <c r="M399" s="7" t="inlineStr"/>
+      <c r="N399" s="7" t="inlineStr"/>
+      <c r="O399" s="7" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="5" t="n">
+        <v>399</v>
+      </c>
+      <c r="B400" s="6" t="inlineStr">
+        <is>
+          <t>online crm</t>
+        </is>
+      </c>
+      <c r="C400" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D400" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E400" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F400" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G400" s="7" t="inlineStr"/>
+      <c r="H400" s="7" t="inlineStr"/>
+      <c r="I400" s="7" t="inlineStr"/>
+      <c r="J400" s="7" t="inlineStr"/>
+      <c r="K400" s="7" t="inlineStr"/>
+      <c r="L400" s="7" t="inlineStr"/>
+      <c r="M400" s="7" t="inlineStr"/>
+      <c r="N400" s="7" t="inlineStr"/>
+      <c r="O400" s="7" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="B401" s="6" t="inlineStr">
+        <is>
+          <t>free crm</t>
+        </is>
+      </c>
+      <c r="C401" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D401" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E401" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F401" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G401" s="7" t="inlineStr"/>
+      <c r="H401" s="7" t="inlineStr"/>
+      <c r="I401" s="7" t="inlineStr"/>
+      <c r="J401" s="7" t="inlineStr"/>
+      <c r="K401" s="7" t="inlineStr"/>
+      <c r="L401" s="7" t="inlineStr"/>
+      <c r="M401" s="7" t="inlineStr"/>
+      <c r="N401" s="7" t="inlineStr"/>
+      <c r="O401" s="7" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="5" t="n">
+        <v>401</v>
+      </c>
+      <c r="B402" s="6" t="inlineStr">
+        <is>
+          <t>best crm</t>
+        </is>
+      </c>
+      <c r="C402" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D402" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E402" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F402" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G402" s="7" t="inlineStr"/>
+      <c r="H402" s="7" t="inlineStr"/>
+      <c r="I402" s="7" t="inlineStr"/>
+      <c r="J402" s="7" t="inlineStr"/>
+      <c r="K402" s="7" t="inlineStr"/>
+      <c r="L402" s="7" t="inlineStr"/>
+      <c r="M402" s="7" t="inlineStr"/>
+      <c r="N402" s="7" t="inlineStr"/>
+      <c r="O402" s="7" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="5" t="n">
+        <v>402</v>
+      </c>
+      <c r="B403" s="6" t="inlineStr">
+        <is>
+          <t>simple crm</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D403" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E403" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F403" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G403" s="7" t="inlineStr"/>
+      <c r="H403" s="7" t="inlineStr"/>
+      <c r="I403" s="7" t="inlineStr"/>
+      <c r="J403" s="7" t="inlineStr"/>
+      <c r="K403" s="7" t="inlineStr"/>
+      <c r="L403" s="7" t="inlineStr"/>
+      <c r="M403" s="7" t="inlineStr"/>
+      <c r="N403" s="7" t="inlineStr"/>
+      <c r="O403" s="7" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="5" t="n">
+        <v>403</v>
+      </c>
+      <c r="B404" s="6" t="inlineStr">
+        <is>
+          <t>crm online</t>
+        </is>
+      </c>
+      <c r="C404" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D404" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E404" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F404" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G404" s="7" t="inlineStr"/>
+      <c r="H404" s="7" t="inlineStr"/>
+      <c r="I404" s="7" t="inlineStr"/>
+      <c r="J404" s="7" t="inlineStr"/>
+      <c r="K404" s="7" t="inlineStr"/>
+      <c r="L404" s="7" t="inlineStr"/>
+      <c r="M404" s="7" t="inlineStr"/>
+      <c r="N404" s="7" t="inlineStr"/>
+      <c r="O404" s="7" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="5" t="n">
+        <v>404</v>
+      </c>
+      <c r="B405" s="6" t="inlineStr">
+        <is>
+          <t>crm for free</t>
+        </is>
+      </c>
+      <c r="C405" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D405" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E405" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F405" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G405" s="7" t="inlineStr"/>
+      <c r="H405" s="7" t="inlineStr"/>
+      <c r="I405" s="7" t="inlineStr"/>
+      <c r="J405" s="7" t="inlineStr"/>
+      <c r="K405" s="7" t="inlineStr"/>
+      <c r="L405" s="7" t="inlineStr"/>
+      <c r="M405" s="7" t="inlineStr"/>
+      <c r="N405" s="7" t="inlineStr"/>
+      <c r="O405" s="7" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="5" t="n">
+        <v>405</v>
+      </c>
+      <c r="B406" s="6" t="inlineStr">
+        <is>
+          <t>crm meaning</t>
+        </is>
+      </c>
+      <c r="C406" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D406" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E406" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F406" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G406" s="7" t="inlineStr"/>
+      <c r="H406" s="7" t="inlineStr"/>
+      <c r="I406" s="7" t="inlineStr"/>
+      <c r="J406" s="7" t="inlineStr"/>
+      <c r="K406" s="7" t="inlineStr"/>
+      <c r="L406" s="7" t="inlineStr"/>
+      <c r="M406" s="7" t="inlineStr"/>
+      <c r="N406" s="7" t="inlineStr"/>
+      <c r="O406" s="7" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="5" t="n">
+        <v>406</v>
+      </c>
+      <c r="B407" s="6" t="inlineStr">
+        <is>
+          <t>what is crm</t>
+        </is>
+      </c>
+      <c r="C407" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D407" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E407" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F407" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G407" s="7" t="inlineStr"/>
+      <c r="H407" s="7" t="inlineStr"/>
+      <c r="I407" s="7" t="inlineStr"/>
+      <c r="J407" s="7" t="inlineStr"/>
+      <c r="K407" s="7" t="inlineStr"/>
+      <c r="L407" s="7" t="inlineStr"/>
+      <c r="M407" s="7" t="inlineStr"/>
+      <c r="N407" s="7" t="inlineStr"/>
+      <c r="O407" s="7" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="5" t="n">
+        <v>407</v>
+      </c>
+      <c r="B408" s="6" t="inlineStr">
+        <is>
+          <t>scheduling app</t>
+        </is>
+      </c>
+      <c r="C408" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D408" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E408" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F408" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G408" s="7" t="inlineStr"/>
+      <c r="H408" s="7" t="inlineStr"/>
+      <c r="I408" s="7" t="inlineStr"/>
+      <c r="J408" s="7" t="inlineStr"/>
+      <c r="K408" s="7" t="inlineStr"/>
+      <c r="L408" s="7" t="inlineStr"/>
+      <c r="M408" s="7" t="inlineStr"/>
+      <c r="N408" s="7" t="inlineStr"/>
+      <c r="O408" s="7" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="5" t="n">
+        <v>408</v>
+      </c>
+      <c r="B409" s="6" t="inlineStr">
+        <is>
+          <t>booking app</t>
+        </is>
+      </c>
+      <c r="C409" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D409" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E409" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F409" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G409" s="7" t="inlineStr"/>
+      <c r="H409" s="7" t="inlineStr"/>
+      <c r="I409" s="7" t="inlineStr"/>
+      <c r="J409" s="7" t="inlineStr"/>
+      <c r="K409" s="7" t="inlineStr"/>
+      <c r="L409" s="7" t="inlineStr"/>
+      <c r="M409" s="7" t="inlineStr"/>
+      <c r="N409" s="7" t="inlineStr"/>
+      <c r="O409" s="7" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="5" t="n">
+        <v>409</v>
+      </c>
+      <c r="B410" s="6" t="inlineStr">
+        <is>
+          <t>invoice app</t>
+        </is>
+      </c>
+      <c r="C410" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D410" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E410" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F410" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G410" s="7" t="inlineStr"/>
+      <c r="H410" s="7" t="inlineStr"/>
+      <c r="I410" s="7" t="inlineStr"/>
+      <c r="J410" s="7" t="inlineStr"/>
+      <c r="K410" s="7" t="inlineStr"/>
+      <c r="L410" s="7" t="inlineStr"/>
+      <c r="M410" s="7" t="inlineStr"/>
+      <c r="N410" s="7" t="inlineStr"/>
+      <c r="O410" s="7" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="B411" s="6" t="inlineStr">
+        <is>
+          <t>invoicing app</t>
+        </is>
+      </c>
+      <c r="C411" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D411" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E411" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F411" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G411" s="7" t="inlineStr"/>
+      <c r="H411" s="7" t="inlineStr"/>
+      <c r="I411" s="7" t="inlineStr"/>
+      <c r="J411" s="7" t="inlineStr"/>
+      <c r="K411" s="7" t="inlineStr"/>
+      <c r="L411" s="7" t="inlineStr"/>
+      <c r="M411" s="7" t="inlineStr"/>
+      <c r="N411" s="7" t="inlineStr"/>
+      <c r="O411" s="7" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="5" t="n">
+        <v>411</v>
+      </c>
+      <c r="B412" s="6" t="inlineStr">
+        <is>
+          <t>free invoicing</t>
+        </is>
+      </c>
+      <c r="C412" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D412" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E412" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F412" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G412" s="7" t="inlineStr"/>
+      <c r="H412" s="7" t="inlineStr"/>
+      <c r="I412" s="7" t="inlineStr"/>
+      <c r="J412" s="7" t="inlineStr"/>
+      <c r="K412" s="7" t="inlineStr"/>
+      <c r="L412" s="7" t="inlineStr"/>
+      <c r="M412" s="7" t="inlineStr"/>
+      <c r="N412" s="7" t="inlineStr"/>
+      <c r="O412" s="7" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="5" t="n">
+        <v>412</v>
+      </c>
+      <c r="B413" s="6" t="inlineStr">
+        <is>
+          <t>best invoicing</t>
+        </is>
+      </c>
+      <c r="C413" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D413" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E413" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F413" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G413" s="7" t="inlineStr"/>
+      <c r="H413" s="7" t="inlineStr"/>
+      <c r="I413" s="7" t="inlineStr"/>
+      <c r="J413" s="7" t="inlineStr"/>
+      <c r="K413" s="7" t="inlineStr"/>
+      <c r="L413" s="7" t="inlineStr"/>
+      <c r="M413" s="7" t="inlineStr"/>
+      <c r="N413" s="7" t="inlineStr"/>
+      <c r="O413" s="7" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="B414" s="6" t="inlineStr">
+        <is>
+          <t>online invoicing</t>
+        </is>
+      </c>
+      <c r="C414" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D414" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E414" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F414" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G414" s="7" t="inlineStr"/>
+      <c r="H414" s="7" t="inlineStr"/>
+      <c r="I414" s="7" t="inlineStr"/>
+      <c r="J414" s="7" t="inlineStr"/>
+      <c r="K414" s="7" t="inlineStr"/>
+      <c r="L414" s="7" t="inlineStr"/>
+      <c r="M414" s="7" t="inlineStr"/>
+      <c r="N414" s="7" t="inlineStr"/>
+      <c r="O414" s="7" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="5" t="n">
+        <v>414</v>
+      </c>
+      <c r="B415" s="6" t="inlineStr">
+        <is>
+          <t>free scheduling app</t>
+        </is>
+      </c>
+      <c r="C415" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D415" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E415" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F415" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G415" s="7" t="inlineStr"/>
+      <c r="H415" s="7" t="inlineStr"/>
+      <c r="I415" s="7" t="inlineStr"/>
+      <c r="J415" s="7" t="inlineStr"/>
+      <c r="K415" s="7" t="inlineStr"/>
+      <c r="L415" s="7" t="inlineStr"/>
+      <c r="M415" s="7" t="inlineStr"/>
+      <c r="N415" s="7" t="inlineStr"/>
+      <c r="O415" s="7" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="5" t="n">
+        <v>415</v>
+      </c>
+      <c r="B416" s="6" t="inlineStr">
+        <is>
+          <t>client management app</t>
+        </is>
+      </c>
+      <c r="C416" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D416" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E416" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F416" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G416" s="7" t="inlineStr"/>
+      <c r="H416" s="7" t="inlineStr"/>
+      <c r="I416" s="7" t="inlineStr"/>
+      <c r="J416" s="7" t="inlineStr"/>
+      <c r="K416" s="7" t="inlineStr"/>
+      <c r="L416" s="7" t="inlineStr"/>
+      <c r="M416" s="7" t="inlineStr"/>
+      <c r="N416" s="7" t="inlineStr"/>
+      <c r="O416" s="7" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="B417" s="6" t="inlineStr">
+        <is>
+          <t>lead tracker</t>
+        </is>
+      </c>
+      <c r="C417" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D417" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E417" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F417" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G417" s="7" t="inlineStr"/>
+      <c r="H417" s="7" t="inlineStr"/>
+      <c r="I417" s="7" t="inlineStr"/>
+      <c r="J417" s="7" t="inlineStr"/>
+      <c r="K417" s="7" t="inlineStr"/>
+      <c r="L417" s="7" t="inlineStr"/>
+      <c r="M417" s="7" t="inlineStr"/>
+      <c r="N417" s="7" t="inlineStr"/>
+      <c r="O417" s="7" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="5" t="n">
+        <v>417</v>
+      </c>
+      <c r="B418" s="6" t="inlineStr">
+        <is>
+          <t>sales tracker</t>
+        </is>
+      </c>
+      <c r="C418" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D418" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E418" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F418" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G418" s="7" t="inlineStr"/>
+      <c r="H418" s="7" t="inlineStr"/>
+      <c r="I418" s="7" t="inlineStr"/>
+      <c r="J418" s="7" t="inlineStr"/>
+      <c r="K418" s="7" t="inlineStr"/>
+      <c r="L418" s="7" t="inlineStr"/>
+      <c r="M418" s="7" t="inlineStr"/>
+      <c r="N418" s="7" t="inlineStr"/>
+      <c r="O418" s="7" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="5" t="n">
+        <v>418</v>
+      </c>
+      <c r="B419" s="6" t="inlineStr">
+        <is>
+          <t>crm software free</t>
+        </is>
+      </c>
+      <c r="C419" s="5" t="inlineStr">
+        <is>
+          <t>Head / short term</t>
+        </is>
+      </c>
+      <c r="D419" s="5" t="inlineStr">
+        <is>
+          <t>All ICPs</t>
+        </is>
+      </c>
+      <c r="E419" s="5" t="inlineStr">
+        <is>
+          <t>Head (short-modifier)</t>
+        </is>
+      </c>
+      <c r="F419" s="5" t="inlineStr">
+        <is>
+          <t>Head (highest volume / broad)</t>
+        </is>
+      </c>
+      <c r="G419" s="7" t="inlineStr"/>
+      <c r="H419" s="7" t="inlineStr"/>
+      <c r="I419" s="7" t="inlineStr"/>
+      <c r="J419" s="7" t="inlineStr"/>
+      <c r="K419" s="7" t="inlineStr"/>
+      <c r="L419" s="7" t="inlineStr"/>
+      <c r="M419" s="7" t="inlineStr"/>
+      <c r="N419" s="7" t="inlineStr"/>
+      <c r="O419" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O352"/>
+  <autoFilter ref="A1:O419"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14405,7 +17018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A368"/>
+  <dimension ref="A1:A437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -16923,6 +19536,481 @@
         </is>
       </c>
     </row>
+    <row r="370">
+      <c r="A370" s="9">
+        <f>== HEAD / SHORT TERMS (67) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>invoicing</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>invoice</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>proposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>appointments</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>quotes</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>helpdesk</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>newsletters</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>contacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>client management</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>project management</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>lead management</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>contact management</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>marketing automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>email marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>appointment scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>online scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>time tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>customer support</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>live chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>client portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>sales pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>task management</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>work management</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>customer onboarding</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>sales tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>deal pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>business management</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>client tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>lead tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>sales automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>email automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>crm app</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>online crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>free crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>best crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>simple crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>crm online</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>crm for free</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>crm meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>what is crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>scheduling app</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>booking app</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>invoice app</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>invoicing app</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>free invoicing</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>best invoicing</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>online invoicing</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>free scheduling app</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>client management app</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>lead tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>sales tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>crm software free</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>